<commit_message>
v1.6.1 — jersey number 0 and 00 (distinct single/double zero); roster template number column as text
- Uniform number picker: add a single "0" on its own first row, before "00";
  selection now distinguishes "0" from "00" (exact match) while legacy un-padded
  imports still select their padded cell.
- displayJersey: keep "0" and "00" verbatim (no longer collapse "0" into "00").
- roster_template.xlsx: format the "number" column as text so "0"/"00" typed in
  Excel survive import instead of being coerced to 0.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/src/main/assets/roster_template.xlsx
+++ b/app/src/main/assets/roster_template.xlsx
@@ -7,12 +7,53 @@
 </workbook>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+  <dxfs count="0"/>
+</styleSheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="16"/>
     <col min="2" max="2" width="10"/>
-    <col min="3" max="3" width="8"/>
+    <col min="3" max="3" width="8" style="1"/>
     <col min="4" max="4" width="12"/>
     <col min="5" max="5" width="12"/>
     <col min="6" max="6" width="26"/>
@@ -29,7 +70,7 @@
           <t xml:space="preserve">gender</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">number</t>
         </is>
@@ -61,7 +102,7 @@
           <t xml:space="preserve">female</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4</t>
         </is>
@@ -93,7 +134,7 @@
           <t xml:space="preserve">female</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">7</t>
         </is>
@@ -125,7 +166,7 @@
           <t xml:space="preserve">male</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">6</t>
         </is>
@@ -157,7 +198,7 @@
           <t xml:space="preserve">female</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">5</t>
         </is>

</xml_diff>